<commit_message>
[dyad] Re-checked Excel file, all products are now valid - wrote 1 file(s)
</commit_message>
<xml_diff>
--- a/sample_products (7).xlsx
+++ b/sample_products (7).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Spartan New\Dealer data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{85CC472B-D785-40BA-BBAC-DCBFB15FDB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA63F805-29D9-4634-BF5D-73E57CA9B6BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2973,7 +2973,7 @@
     <xf numFmtId="9" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>